<commit_message>
Excel: malzeme satırları I:J birleştirme tutarlılığı + Plastik Kasa satırı
- Şablonda 16,18,19,20,21,22,24. satırlarda eksik olan I:J hücre
  birleştirmesi eklendi (kullanıcının elle düzenlediği dosyayla eşleşecek
  şekilde, malzeme alanındaki tüm satırlar artık tutarlı).
- record_excel_template.php: malzeme listesinin hemen altına, gerçek bir
  malzeme tanımı olmayan "PLASTİK KASA" satırı otomatik ekleniyor —
  K sütunu canlı =O13 formülüyle TOPLAM KASA ADETİ'ni birebir yansıtıyor.
- Sürüm v177 (sw.js CACHE_NAME + APP_SURUM + CLAUDE.md).
</commit_message>
<xml_diff>
--- a/templates/excel/yukleme_plani_template.xlsx
+++ b/templates/excel/yukleme_plani_template.xlsx
@@ -2203,6 +2203,13 @@
     <mergeCell ref="O32:P32"/>
     <mergeCell ref="I33:J33"/>
     <mergeCell ref="O33:P33"/>
+    <mergeCell ref="I16:J16"/>
+    <mergeCell ref="I18:J18"/>
+    <mergeCell ref="I19:J19"/>
+    <mergeCell ref="I20:J20"/>
+    <mergeCell ref="I21:J21"/>
+    <mergeCell ref="I22:J22"/>
+    <mergeCell ref="I24:J24"/>
   </mergeCells>
   <printOptions gridLines="false" gridLinesSet="true"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>